<commit_message>
Revert "finalize Aim2 primary"
This reverts commit 604768805506fae1f32bc5c64cb0385e813ca336.
</commit_message>
<xml_diff>
--- a/code/Table_aim2_secondary.xlsx
+++ b/code/Table_aim2_secondary.xlsx
@@ -439,13 +439,13 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
     <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="22" customWidth="1" min="17" max="17"/>
-    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
     <col width="19" customWidth="1" min="19" max="19"/>
     <col width="22" customWidth="1" min="20" max="20"/>
     <col width="19" customWidth="1" min="21" max="21"/>
@@ -641,43 +641,43 @@
         <v>28</v>
       </c>
       <c r="K2" t="n">
-        <v>1.483193421444162</v>
+        <v>0.1300873374734078</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1524771781316907</v>
+        <v>0.08817329002033837</v>
       </c>
       <c r="M2" t="n">
-        <v>1.39820636722879</v>
+        <v>0.09856125657661254</v>
       </c>
       <c r="N2" t="n">
-        <v>0.2064492702701683</v>
+        <v>0.05640396151733591</v>
       </c>
       <c r="O2" t="n">
-        <v>0.08498705421537256</v>
+        <v>0.03152608089679527</v>
       </c>
       <c r="P2" t="n">
-        <v>0.4614252999197991</v>
+        <v>0.4353656622096378</v>
       </c>
       <c r="Q2" t="n">
-        <v>-0.06400202764473212</v>
+        <v>-0.1495200746536932</v>
       </c>
       <c r="R2" t="n">
-        <v>0.9722754614838974</v>
+        <v>1.004943824017964</v>
       </c>
       <c r="S2" t="n">
         <v>5000</v>
       </c>
       <c r="T2" t="n">
-        <v>1.688623307581887</v>
+        <v>1.483445301774754</v>
       </c>
       <c r="U2" t="n">
-        <v>48.51142280322171</v>
+        <v>35.96466015948098</v>
       </c>
       <c r="V2" t="n">
-        <v>0.09771068060853218</v>
+        <v>0.1466675369782948</v>
       </c>
       <c r="W2" t="n">
-        <v>0.1727977323906871</v>
+        <v>0.3422242529493546</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -747,47 +747,47 @@
         <v>28</v>
       </c>
       <c r="K3" t="n">
-        <v>1.479823626483557</v>
+        <v>0.1285551021579494</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1942086984353445</v>
+        <v>0.09264756978923594</v>
       </c>
       <c r="M3" t="n">
-        <v>1.558473712815117</v>
+        <v>0.1267838346433344</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1195652140947562</v>
+        <v>0.09698240949272487</v>
       </c>
       <c r="O3" t="n">
-        <v>-0.07865008633156001</v>
+        <v>0.001771267514614983</v>
       </c>
       <c r="P3" t="n">
-        <v>-0.4993130805700229</v>
+        <v>0.01863303336686996</v>
       </c>
       <c r="Q3" t="n">
-        <v>-0.9740859627007233</v>
+        <v>-0.513565675083519</v>
       </c>
       <c r="R3" t="n">
-        <v>0.02346077765077016</v>
+        <v>0.5922022128950996</v>
       </c>
       <c r="S3" t="n">
         <v>5000</v>
       </c>
       <c r="T3" t="n">
-        <v>-1.696039382747858</v>
+        <v>0.06651606431530295</v>
       </c>
       <c r="U3" t="n">
-        <v>35.06238254286284</v>
+        <v>47.84413069520072</v>
       </c>
       <c r="V3" t="n">
-        <v>0.09874156136610693</v>
+        <v>0.9472441508466121</v>
       </c>
       <c r="W3" t="n">
-        <v>0.1727977323906871</v>
+        <v>0.9472441508466121</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>lower in SAD</t>
+          <t>higher in SAD</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -853,47 +853,47 @@
         <v>28</v>
       </c>
       <c r="K4" t="n">
-        <v>1.517341694840898</v>
+        <v>0.1783705426639688</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1198274062129216</v>
+        <v>0.1269747265245408</v>
       </c>
       <c r="M4" t="n">
-        <v>1.519858740961526</v>
+        <v>0.1366094902291264</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1317298784074646</v>
+        <v>0.1171885142545761</v>
       </c>
       <c r="O4" t="n">
-        <v>-0.00251704612062742</v>
+        <v>0.04176105243484235</v>
       </c>
       <c r="P4" t="n">
-        <v>-0.01989374615125264</v>
+        <v>0.3432047005582242</v>
       </c>
       <c r="Q4" t="n">
-        <v>-0.6127509058360042</v>
+        <v>-0.1970101615398488</v>
       </c>
       <c r="R4" t="n">
-        <v>0.5247360362081663</v>
+        <v>0.9713910618300602</v>
       </c>
       <c r="S4" t="n">
         <v>5000</v>
       </c>
       <c r="T4" t="n">
-        <v>-0.07136347141985432</v>
+        <v>1.209854869467374</v>
       </c>
       <c r="U4" t="n">
-        <v>48.45301578991505</v>
+        <v>45.4332277238017</v>
       </c>
       <c r="V4" t="n">
-        <v>0.9434022332141585</v>
+        <v>0.2325921056656618</v>
       </c>
       <c r="W4" t="n">
-        <v>0.9434022332141585</v>
+        <v>0.4070361849149082</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>lower in SAD</t>
+          <t>higher in SAD</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -1204,7 +1204,7 @@
         <v>0.9343969974782784</v>
       </c>
       <c r="W7" t="n">
-        <v>0.9434022332141585</v>
+        <v>0.9472441508466121</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
upate the hyak workflow
</commit_message>
<xml_diff>
--- a/code/Table_aim2_secondary.xlsx
+++ b/code/Table_aim2_secondary.xlsx
@@ -439,7 +439,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
@@ -641,43 +641,43 @@
         <v>28</v>
       </c>
       <c r="K2" t="n">
-        <v>0.1300873374734078</v>
+        <v>0.2314684506042999</v>
       </c>
       <c r="L2" t="n">
-        <v>0.08817329002033837</v>
+        <v>0.1533706281069297</v>
       </c>
       <c r="M2" t="n">
-        <v>0.09856125657661254</v>
+        <v>0.2074879754890014</v>
       </c>
       <c r="N2" t="n">
-        <v>0.05640396151733591</v>
+        <v>0.1310787385108941</v>
       </c>
       <c r="O2" t="n">
-        <v>0.03152608089679527</v>
+        <v>0.02398047511529852</v>
       </c>
       <c r="P2" t="n">
-        <v>0.4353656622096378</v>
+        <v>0.1694465536944773</v>
       </c>
       <c r="Q2" t="n">
-        <v>-0.1495200746536932</v>
+        <v>-0.3961783266510094</v>
       </c>
       <c r="R2" t="n">
-        <v>1.004943824017964</v>
+        <v>0.7290540536252698</v>
       </c>
       <c r="S2" t="n">
         <v>5000</v>
       </c>
       <c r="T2" t="n">
-        <v>1.483445301774754</v>
+        <v>0.5928157910303914</v>
       </c>
       <c r="U2" t="n">
-        <v>35.96466015948098</v>
+        <v>43.54635217281516</v>
       </c>
       <c r="V2" t="n">
-        <v>0.1466675369782948</v>
+        <v>0.5563707173345738</v>
       </c>
       <c r="W2" t="n">
-        <v>0.3422242529493546</v>
+        <v>0.6517481117828272</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -747,43 +747,43 @@
         <v>28</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1285551021579494</v>
+        <v>0.250406860425123</v>
       </c>
       <c r="L3" t="n">
-        <v>0.09264756978923594</v>
+        <v>0.1177094810781026</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1267838346433344</v>
+        <v>0.2302064012448476</v>
       </c>
       <c r="N3" t="n">
-        <v>0.09698240949272487</v>
+        <v>0.1267753928149779</v>
       </c>
       <c r="O3" t="n">
-        <v>0.001771267514614983</v>
+        <v>0.02020045918027544</v>
       </c>
       <c r="P3" t="n">
-        <v>0.01863303336686996</v>
+        <v>0.1645151819033414</v>
       </c>
       <c r="Q3" t="n">
-        <v>-0.513565675083519</v>
+        <v>-0.3872726190506065</v>
       </c>
       <c r="R3" t="n">
-        <v>0.5922022128950996</v>
+        <v>0.7627129097762194</v>
       </c>
       <c r="S3" t="n">
         <v>5000</v>
       </c>
       <c r="T3" t="n">
-        <v>0.06651606431530295</v>
+        <v>0.5889536918794687</v>
       </c>
       <c r="U3" t="n">
-        <v>47.84413069520072</v>
+        <v>48.22395824619176</v>
       </c>
       <c r="V3" t="n">
-        <v>0.9472441508466121</v>
+        <v>0.5586412386709947</v>
       </c>
       <c r="W3" t="n">
-        <v>0.9472441508466121</v>
+        <v>0.6517481117828272</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -853,43 +853,43 @@
         <v>28</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1783705426639688</v>
+        <v>0.2991152799714809</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1269747265245408</v>
+        <v>0.1760392869776785</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1366094902291264</v>
+        <v>0.239382628137274</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1171885142545761</v>
+        <v>0.1424927437816819</v>
       </c>
       <c r="O4" t="n">
-        <v>0.04176105243484235</v>
+        <v>0.05973265183420687</v>
       </c>
       <c r="P4" t="n">
-        <v>0.3432047005582242</v>
+        <v>0.3770154856650065</v>
       </c>
       <c r="Q4" t="n">
-        <v>-0.1970101615398488</v>
+        <v>-0.1819640990020789</v>
       </c>
       <c r="R4" t="n">
-        <v>0.9713910618300602</v>
+        <v>0.9446261346784078</v>
       </c>
       <c r="S4" t="n">
         <v>5000</v>
       </c>
       <c r="T4" t="n">
-        <v>1.209854869467374</v>
+        <v>1.31208218114335</v>
       </c>
       <c r="U4" t="n">
-        <v>45.4332277238017</v>
+        <v>42.11345390330619</v>
       </c>
       <c r="V4" t="n">
-        <v>0.2325921056656618</v>
+        <v>0.1965995474682463</v>
       </c>
       <c r="W4" t="n">
-        <v>0.4070361849149082</v>
+        <v>0.4587322774259079</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -1204,7 +1204,7 @@
         <v>0.9343969974782784</v>
       </c>
       <c r="W7" t="n">
-        <v>0.9472441508466121</v>
+        <v>0.9343969974782784</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
@@ -1309,7 +1309,7 @@
         <v>0.3322741430099554</v>
       </c>
       <c r="W8" t="n">
-        <v>0.4651838002139375</v>
+        <v>0.5814797502674219</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>

</xml_diff>